<commit_message>
Add data cleaning and clustering analysis for production data
</commit_message>
<xml_diff>
--- a/data/sample/DailyProductionReport_17032026.xlsx
+++ b/data/sample/DailyProductionReport_17032026.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VARSHA\FactorDataReconcilation\essenn-production-vs-plan\data\sample\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50CFB45E-C296-488E-A6B7-1060E0A342FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="132" yWindow="564" windowWidth="30396" windowHeight="13164"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3154,7 +3160,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3">
     <font>
       <sz val="11"/>
@@ -3293,29 +3299,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="9">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3324,13 +3330,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3368,7 +3382,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -3402,6 +3416,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -3436,9 +3451,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3611,27 +3627,27 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S566"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="15" style="1" customWidth="1"/>
     <col min="2" max="2" width="17.44140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="35" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9.109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="15.44140625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="12" style="1" customWidth="1"/>
+    <col min="4" max="4" width="39.109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="26.5546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="34.6640625" style="1" customWidth="1"/>
     <col min="7" max="7" width="21.109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="9.109375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="13.44140625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="15" style="1" customWidth="1"/>
+    <col min="9" max="9" width="32.44140625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="27.109375" style="1" customWidth="1"/>
     <col min="11" max="11" width="10.6640625" style="1" customWidth="1"/>
     <col min="12" max="12" width="15.5546875" style="1" customWidth="1"/>
     <col min="13" max="13" width="10" style="1" customWidth="1"/>
     <col min="14" max="14" width="15.21875" style="1" customWidth="1"/>
     <col min="15" max="15" width="21.33203125" style="1" customWidth="1"/>
     <col min="16" max="16" width="11.5546875" style="1" customWidth="1"/>
-    <col min="17" max="17" width="23.5546875" style="1" customWidth="1"/>
+    <col min="17" max="17" width="85.6640625" style="1" customWidth="1"/>
     <col min="18" max="18" width="19.33203125" style="1" customWidth="1"/>
     <col min="19" max="20" width="9.109375" style="1" customWidth="1"/>
     <col min="21" max="16384" width="9.109375" style="1"/>
@@ -37032,7 +37048,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S566"/>
+  <autoFilter ref="A1:S566" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>